<commit_message>
Versione 2: aggiornamenti vari, Aggiunto smistamento file scarico locale a caricamento file anteprima -donload
</commit_message>
<xml_diff>
--- a/elenco_codici_studi.xlsx
+++ b/elenco_codici_studi.xlsx
@@ -23719,6 +23719,11 @@
           <t>T35P060</t>
         </is>
       </c>
+      <c r="B2346" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2347">
       <c r="A2347" t="inlineStr">
@@ -23796,6 +23801,11 @@
           <t>T35P071</t>
         </is>
       </c>
+      <c r="B2357" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2358">
       <c r="A2358" t="inlineStr">
@@ -23803,6 +23813,11 @@
           <t>T35P072</t>
         </is>
       </c>
+      <c r="B2358" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2359">
       <c r="A2359" t="inlineStr">
@@ -23894,6 +23909,11 @@
           <t>T35P085</t>
         </is>
       </c>
+      <c r="B2371" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2372">
       <c r="A2372" t="inlineStr">
@@ -23901,6 +23921,11 @@
           <t>T35P086</t>
         </is>
       </c>
+      <c r="B2372" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2373">
       <c r="A2373" t="inlineStr">
@@ -23908,6 +23933,11 @@
           <t>T35P087</t>
         </is>
       </c>
+      <c r="B2373" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2374">
       <c r="A2374" t="inlineStr">
@@ -23915,6 +23945,11 @@
           <t>T35P088</t>
         </is>
       </c>
+      <c r="B2374" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2375">
       <c r="A2375" t="inlineStr">
@@ -23922,6 +23957,11 @@
           <t>T35P089</t>
         </is>
       </c>
+      <c r="B2375" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2376">
       <c r="A2376" t="inlineStr">
@@ -23929,6 +23969,11 @@
           <t>T35P090</t>
         </is>
       </c>
+      <c r="B2376" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2377">
       <c r="A2377" t="inlineStr">
@@ -23936,6 +23981,11 @@
           <t>T35P091</t>
         </is>
       </c>
+      <c r="B2377" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2378">
       <c r="A2378" t="inlineStr">
@@ -23943,6 +23993,11 @@
           <t>T35P092</t>
         </is>
       </c>
+      <c r="B2378" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2379">
       <c r="A2379" t="inlineStr">
@@ -23950,6 +24005,11 @@
           <t>T35P093</t>
         </is>
       </c>
+      <c r="B2379" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2380">
       <c r="A2380" t="inlineStr">
@@ -23957,6 +24017,11 @@
           <t>T35P094</t>
         </is>
       </c>
+      <c r="B2380" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2381">
       <c r="A2381" t="inlineStr">
@@ -23964,6 +24029,11 @@
           <t>T35P095</t>
         </is>
       </c>
+      <c r="B2381" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2382">
       <c r="A2382" t="inlineStr">
@@ -23971,6 +24041,11 @@
           <t>T35P096</t>
         </is>
       </c>
+      <c r="B2382" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2383">
       <c r="A2383" t="inlineStr">
@@ -23978,6 +24053,11 @@
           <t>T35P097</t>
         </is>
       </c>
+      <c r="B2383" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2384">
       <c r="A2384" t="inlineStr">
@@ -23985,6 +24065,11 @@
           <t>T35P098</t>
         </is>
       </c>
+      <c r="B2384" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2385">
       <c r="A2385" t="inlineStr">
@@ -23992,6 +24077,11 @@
           <t>T35P099</t>
         </is>
       </c>
+      <c r="B2385" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2386">
       <c r="A2386" t="inlineStr">
@@ -23999,6 +24089,11 @@
           <t>T35P100</t>
         </is>
       </c>
+      <c r="B2386" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2387">
       <c r="A2387" t="inlineStr">
@@ -24006,6 +24101,11 @@
           <t>T35P101</t>
         </is>
       </c>
+      <c r="B2387" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2388">
       <c r="A2388" t="inlineStr">
@@ -24013,6 +24113,11 @@
           <t>T35P103</t>
         </is>
       </c>
+      <c r="B2388" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2389">
       <c r="A2389" t="inlineStr">
@@ -24104,6 +24209,11 @@
           <t>T3AP013</t>
         </is>
       </c>
+      <c r="B2401" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2402">
       <c r="A2402" t="inlineStr">
@@ -24111,6 +24221,11 @@
           <t>T3AP014</t>
         </is>
       </c>
+      <c r="B2402" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2403">
       <c r="A2403" t="inlineStr">
@@ -24118,6 +24233,11 @@
           <t>T3AP015</t>
         </is>
       </c>
+      <c r="B2403" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2404">
       <c r="A2404" t="inlineStr">
@@ -24125,6 +24245,11 @@
           <t>T3AP016</t>
         </is>
       </c>
+      <c r="B2404" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2405">
       <c r="A2405" t="inlineStr">
@@ -24132,6 +24257,11 @@
           <t>T3AP017</t>
         </is>
       </c>
+      <c r="B2405" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2406">
       <c r="A2406" t="inlineStr">
@@ -24139,6 +24269,11 @@
           <t>T3AP018</t>
         </is>
       </c>
+      <c r="B2406" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2407">
       <c r="A2407" t="inlineStr">
@@ -24195,6 +24330,11 @@
           <t>T3D3012</t>
         </is>
       </c>
+      <c r="B2414" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2415">
       <c r="A2415" t="inlineStr">
@@ -24209,6 +24349,11 @@
           <t>T3K2001</t>
         </is>
       </c>
+      <c r="B2416" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2417">
       <c r="A2417" t="inlineStr">
@@ -24398,6 +24543,11 @@
           <t>T3K2039</t>
         </is>
       </c>
+      <c r="B2443" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2444">
       <c r="A2444" t="inlineStr">
@@ -24405,6 +24555,11 @@
           <t>T3K2041</t>
         </is>
       </c>
+      <c r="B2444" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2445">
       <c r="A2445" t="inlineStr">
@@ -24412,6 +24567,11 @@
           <t>T3K2042</t>
         </is>
       </c>
+      <c r="B2445" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2446">
       <c r="A2446" t="inlineStr">
@@ -24419,6 +24579,11 @@
           <t>T3K2043</t>
         </is>
       </c>
+      <c r="B2446" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2447">
       <c r="A2447" t="inlineStr">
@@ -24426,6 +24591,11 @@
           <t>T3K2044</t>
         </is>
       </c>
+      <c r="B2447" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2448">
       <c r="A2448" t="inlineStr">
@@ -24433,6 +24603,11 @@
           <t>T3K2045</t>
         </is>
       </c>
+      <c r="B2448" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2449">
       <c r="A2449" t="inlineStr">
@@ -24440,6 +24615,11 @@
           <t>T3K2046</t>
         </is>
       </c>
+      <c r="B2449" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2450">
       <c r="A2450" t="inlineStr">
@@ -24447,6 +24627,11 @@
           <t>T3K2047</t>
         </is>
       </c>
+      <c r="B2450" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2451">
       <c r="A2451" t="inlineStr">
@@ -24454,6 +24639,11 @@
           <t>T3K2048</t>
         </is>
       </c>
+      <c r="B2451" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2452">
       <c r="A2452" t="inlineStr">
@@ -24461,6 +24651,11 @@
           <t>T3K2049</t>
         </is>
       </c>
+      <c r="B2452" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2453">
       <c r="A2453" t="inlineStr">
@@ -24468,6 +24663,11 @@
           <t>T3K2050</t>
         </is>
       </c>
+      <c r="B2453" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2454">
       <c r="A2454" t="inlineStr">
@@ -24475,6 +24675,11 @@
           <t>T3K2051</t>
         </is>
       </c>
+      <c r="B2454" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2455">
       <c r="A2455" t="inlineStr">
@@ -24482,6 +24687,11 @@
           <t>T3K2052</t>
         </is>
       </c>
+      <c r="B2455" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2456">
       <c r="A2456" t="inlineStr">
@@ -24489,6 +24699,11 @@
           <t>T3K2053</t>
         </is>
       </c>
+      <c r="B2456" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2457">
       <c r="A2457" t="inlineStr">
@@ -24496,6 +24711,11 @@
           <t>T3K2054</t>
         </is>
       </c>
+      <c r="B2457" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2458">
       <c r="A2458" t="inlineStr">
@@ -24503,6 +24723,11 @@
           <t>T3K2055</t>
         </is>
       </c>
+      <c r="B2458" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2459">
       <c r="A2459" t="inlineStr">
@@ -24510,6 +24735,11 @@
           <t>T3K2056</t>
         </is>
       </c>
+      <c r="B2459" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2460">
       <c r="A2460" t="inlineStr">
@@ -24517,6 +24747,11 @@
           <t>T3K2057</t>
         </is>
       </c>
+      <c r="B2460" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2461">
       <c r="A2461" t="inlineStr">
@@ -24524,6 +24759,11 @@
           <t>T3K2058</t>
         </is>
       </c>
+      <c r="B2461" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2462">
       <c r="A2462" t="inlineStr">
@@ -24531,6 +24771,11 @@
           <t>T3K2059</t>
         </is>
       </c>
+      <c r="B2462" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2463">
       <c r="A2463" t="inlineStr">
@@ -24538,6 +24783,11 @@
           <t>T3K2060</t>
         </is>
       </c>
+      <c r="B2463" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2464">
       <c r="A2464" t="inlineStr">
@@ -24545,6 +24795,11 @@
           <t>T3K2061</t>
         </is>
       </c>
+      <c r="B2464" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2465">
       <c r="A2465" t="inlineStr">
@@ -24552,6 +24807,11 @@
           <t>T3K2062</t>
         </is>
       </c>
+      <c r="B2465" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2466">
       <c r="A2466" t="inlineStr">
@@ -24559,6 +24819,11 @@
           <t>T3K2063</t>
         </is>
       </c>
+      <c r="B2466" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2467">
       <c r="A2467" t="inlineStr">
@@ -24566,6 +24831,11 @@
           <t>T3K2064</t>
         </is>
       </c>
+      <c r="B2467" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2468">
       <c r="A2468" t="inlineStr">
@@ -24573,6 +24843,11 @@
           <t>T3K2065</t>
         </is>
       </c>
+      <c r="B2468" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2469">
       <c r="A2469" t="inlineStr">
@@ -24587,6 +24862,11 @@
           <t>T40P002</t>
         </is>
       </c>
+      <c r="B2470" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2471">
       <c r="A2471" t="inlineStr">
@@ -24594,6 +24874,11 @@
           <t>T40P003</t>
         </is>
       </c>
+      <c r="B2471" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2472">
       <c r="A2472" t="inlineStr">
@@ -24601,6 +24886,11 @@
           <t>T40P005</t>
         </is>
       </c>
+      <c r="B2472" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2473">
       <c r="A2473" t="inlineStr">
@@ -24608,6 +24898,11 @@
           <t>T40P009</t>
         </is>
       </c>
+      <c r="B2473" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2474">
       <c r="A2474" t="inlineStr">
@@ -24615,6 +24910,11 @@
           <t>T40P010</t>
         </is>
       </c>
+      <c r="B2474" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2475">
       <c r="A2475" t="inlineStr">
@@ -24643,6 +24943,11 @@
           <t>T40P015</t>
         </is>
       </c>
+      <c r="B2478" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2479">
       <c r="A2479" t="inlineStr">
@@ -24664,6 +24969,11 @@
           <t>T40P019</t>
         </is>
       </c>
+      <c r="B2481" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2482">
       <c r="A2482" t="inlineStr">
@@ -24671,6 +24981,11 @@
           <t>T450001</t>
         </is>
       </c>
+      <c r="B2482" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2483">
       <c r="A2483" t="inlineStr">
@@ -24678,6 +24993,11 @@
           <t>T450002</t>
         </is>
       </c>
+      <c r="B2483" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2484">
       <c r="A2484" t="inlineStr">
@@ -24685,6 +25005,11 @@
           <t>T450003</t>
         </is>
       </c>
+      <c r="B2484" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2485">
       <c r="A2485" t="inlineStr">
@@ -24692,6 +25017,11 @@
           <t>T450004</t>
         </is>
       </c>
+      <c r="B2485" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2486">
       <c r="A2486" t="inlineStr">
@@ -24748,6 +25078,11 @@
           <t>T90P007</t>
         </is>
       </c>
+      <c r="B2493" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2494">
       <c r="A2494" t="inlineStr">
@@ -24755,6 +25090,11 @@
           <t>T90P008</t>
         </is>
       </c>
+      <c r="B2494" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2495">
       <c r="A2495" t="inlineStr">
@@ -24762,6 +25102,11 @@
           <t>T90P009</t>
         </is>
       </c>
+      <c r="B2495" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2496">
       <c r="A2496" t="inlineStr">
@@ -24769,6 +25114,11 @@
           <t>T90P010</t>
         </is>
       </c>
+      <c r="B2496" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2497">
       <c r="A2497" t="inlineStr">
@@ -24776,6 +25126,11 @@
           <t>TGLO003</t>
         </is>
       </c>
+      <c r="B2497" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2498">
       <c r="A2498" t="inlineStr">
@@ -24783,6 +25138,11 @@
           <t>TGLO004</t>
         </is>
       </c>
+      <c r="B2498" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2499">
       <c r="A2499" t="inlineStr">
@@ -24790,6 +25150,11 @@
           <t>TGLO005</t>
         </is>
       </c>
+      <c r="B2499" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2500">
       <c r="A2500" t="inlineStr">
@@ -24797,6 +25162,11 @@
           <t>TMXE001</t>
         </is>
       </c>
+      <c r="B2500" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2501">
       <c r="A2501" t="inlineStr">
@@ -24804,6 +25174,11 @@
           <t>TMXE002</t>
         </is>
       </c>
+      <c r="B2501" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2502">
       <c r="A2502" t="inlineStr">
@@ -24818,6 +25193,11 @@
           <t>TMXE037</t>
         </is>
       </c>
+      <c r="B2503" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2504">
       <c r="A2504" t="inlineStr">
@@ -24860,6 +25240,11 @@
           <t>TMXE044</t>
         </is>
       </c>
+      <c r="B2509" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2510">
       <c r="A2510" t="inlineStr">
@@ -24867,6 +25252,11 @@
           <t>TMXE045</t>
         </is>
       </c>
+      <c r="B2510" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2511">
       <c r="A2511" t="inlineStr">
@@ -24874,6 +25264,11 @@
           <t>TMXE046</t>
         </is>
       </c>
+      <c r="B2511" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2512">
       <c r="A2512" t="inlineStr">
@@ -24881,6 +25276,11 @@
           <t>TMXE047</t>
         </is>
       </c>
+      <c r="B2512" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2513">
       <c r="A2513" t="inlineStr">
@@ -24888,6 +25288,11 @@
           <t>TNDM002</t>
         </is>
       </c>
+      <c r="B2513" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2514">
       <c r="A2514" t="inlineStr">
@@ -24895,6 +25300,11 @@
           <t>TRT1001</t>
         </is>
       </c>
+      <c r="B2514" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2515">
       <c r="A2515" t="inlineStr">
@@ -24902,6 +25312,11 @@
           <t>TRT1002</t>
         </is>
       </c>
+      <c r="B2515" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2516">
       <c r="A2516" t="inlineStr">
@@ -24909,6 +25324,11 @@
           <t>TRT1003</t>
         </is>
       </c>
+      <c r="B2516" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2517">
       <c r="A2517" t="inlineStr">
@@ -24916,6 +25336,11 @@
           <t>TRT1004</t>
         </is>
       </c>
+      <c r="B2517" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2518">
       <c r="A2518" t="inlineStr">
@@ -24923,6 +25348,11 @@
           <t>TRT1005</t>
         </is>
       </c>
+      <c r="B2518" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2519">
       <c r="A2519" t="inlineStr">
@@ -24930,6 +25360,11 @@
           <t>TRT1006</t>
         </is>
       </c>
+      <c r="B2519" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2520">
       <c r="A2520" t="inlineStr">
@@ -24937,6 +25372,11 @@
           <t>TS10001</t>
         </is>
       </c>
+      <c r="B2520" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2521">
       <c r="A2521" t="inlineStr">
@@ -24951,6 +25391,11 @@
           <t>TS10004</t>
         </is>
       </c>
+      <c r="B2522" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2523">
       <c r="A2523" t="inlineStr">
@@ -24958,6 +25403,11 @@
           <t>TS10005</t>
         </is>
       </c>
+      <c r="B2523" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2524">
       <c r="A2524" t="inlineStr">
@@ -24965,6 +25415,11 @@
           <t>TS10006</t>
         </is>
       </c>
+      <c r="B2524" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2525">
       <c r="A2525" t="inlineStr">
@@ -24972,6 +25427,11 @@
           <t>TS10008</t>
         </is>
       </c>
+      <c r="B2525" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2526">
       <c r="A2526" t="inlineStr">
@@ -24979,6 +25439,11 @@
           <t>TS10009</t>
         </is>
       </c>
+      <c r="B2526" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2527">
       <c r="A2527" t="inlineStr">
@@ -24986,6 +25451,11 @@
           <t>TS10010</t>
         </is>
       </c>
+      <c r="B2527" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2528">
       <c r="A2528" t="inlineStr">
@@ -24993,6 +25463,11 @@
           <t>TS10011</t>
         </is>
       </c>
+      <c r="B2528" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2529">
       <c r="A2529" t="inlineStr">
@@ -25000,6 +25475,11 @@
           <t>TT10002</t>
         </is>
       </c>
+      <c r="B2529" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2530">
       <c r="A2530" t="inlineStr">
@@ -25007,6 +25487,11 @@
           <t>TT30001</t>
         </is>
       </c>
+      <c r="B2530" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2531">
       <c r="A2531" t="inlineStr">
@@ -25014,6 +25499,11 @@
           <t>TT30002</t>
         </is>
       </c>
+      <c r="B2531" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2532">
       <c r="A2532" t="inlineStr">
@@ -25021,6 +25511,11 @@
           <t>TT30003</t>
         </is>
       </c>
+      <c r="B2532" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2533">
       <c r="A2533" t="inlineStr">
@@ -25028,6 +25523,11 @@
           <t>TT30004</t>
         </is>
       </c>
+      <c r="B2533" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2534">
       <c r="A2534" t="inlineStr">
@@ -25035,6 +25535,11 @@
           <t>TT30005</t>
         </is>
       </c>
+      <c r="B2534" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2535">
       <c r="A2535" t="inlineStr">
@@ -25042,6 +25547,11 @@
           <t>TT30006</t>
         </is>
       </c>
+      <c r="B2535" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2536">
       <c r="A2536" t="inlineStr">
@@ -25049,6 +25559,11 @@
           <t>TT30007</t>
         </is>
       </c>
+      <c r="B2536" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2537">
       <c r="A2537" t="inlineStr">
@@ -25056,6 +25571,11 @@
           <t>TT30008</t>
         </is>
       </c>
+      <c r="B2537" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2538">
       <c r="A2538" t="inlineStr">
@@ -25070,6 +25590,11 @@
           <t>TUNI002</t>
         </is>
       </c>
+      <c r="B2539" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2540">
       <c r="A2540" t="inlineStr">
@@ -25077,6 +25602,11 @@
           <t>TUNI003</t>
         </is>
       </c>
+      <c r="B2540" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2541">
       <c r="A2541" t="inlineStr">
@@ -25140,6 +25670,11 @@
           <t>TUNI015</t>
         </is>
       </c>
+      <c r="B2549" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2550">
       <c r="A2550" t="inlineStr">
@@ -25147,6 +25682,11 @@
           <t>TUNI016</t>
         </is>
       </c>
+      <c r="B2550" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2551">
       <c r="A2551" t="inlineStr">
@@ -25168,6 +25708,11 @@
           <t>TUNI019</t>
         </is>
       </c>
+      <c r="B2553" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2554">
       <c r="A2554" t="inlineStr">
@@ -25189,6 +25734,11 @@
           <t>TUNI022</t>
         </is>
       </c>
+      <c r="B2556" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2557">
       <c r="A2557" t="inlineStr">
@@ -25203,6 +25753,11 @@
           <t>TUNI026</t>
         </is>
       </c>
+      <c r="B2558" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2559">
       <c r="A2559" t="inlineStr">
@@ -25231,6 +25786,11 @@
           <t>TUNI031</t>
         </is>
       </c>
+      <c r="B2562" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2563">
       <c r="A2563" t="inlineStr">
@@ -25238,6 +25798,11 @@
           <t>TUNI032</t>
         </is>
       </c>
+      <c r="B2563" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2564">
       <c r="A2564" t="inlineStr">
@@ -25245,6 +25810,11 @@
           <t>TUNI033</t>
         </is>
       </c>
+      <c r="B2564" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2565">
       <c r="A2565" t="inlineStr">
@@ -25252,6 +25822,11 @@
           <t>TUNI034</t>
         </is>
       </c>
+      <c r="B2565" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2566">
       <c r="A2566" t="inlineStr">
@@ -25259,6 +25834,11 @@
           <t>TUNI035</t>
         </is>
       </c>
+      <c r="B2566" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2567">
       <c r="A2567" t="inlineStr">
@@ -25266,6 +25846,11 @@
           <t>TUNI036</t>
         </is>
       </c>
+      <c r="B2567" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2568">
       <c r="A2568" t="inlineStr">
@@ -25273,6 +25858,11 @@
           <t>TUNI037</t>
         </is>
       </c>
+      <c r="B2568" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2569">
       <c r="A2569" t="inlineStr">
@@ -25280,6 +25870,11 @@
           <t>TUNI038</t>
         </is>
       </c>
+      <c r="B2569" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2570">
       <c r="A2570" t="inlineStr">
@@ -25287,6 +25882,11 @@
           <t>TUNI039</t>
         </is>
       </c>
+      <c r="B2570" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2571">
       <c r="A2571" t="inlineStr">
@@ -25294,6 +25894,11 @@
           <t>TUNI040</t>
         </is>
       </c>
+      <c r="B2571" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2572">
       <c r="A2572" t="inlineStr">
@@ -25301,6 +25906,11 @@
           <t>TUNI041</t>
         </is>
       </c>
+      <c r="B2572" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2573">
       <c r="A2573" t="inlineStr">
@@ -25308,6 +25918,11 @@
           <t>TUNI043</t>
         </is>
       </c>
+      <c r="B2573" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2574">
       <c r="A2574" t="inlineStr">
@@ -25315,6 +25930,11 @@
           <t>TUNI045</t>
         </is>
       </c>
+      <c r="B2574" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2575">
       <c r="A2575" t="inlineStr">
@@ -25322,6 +25942,11 @@
           <t>TUNI046</t>
         </is>
       </c>
+      <c r="B2575" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2576">
       <c r="A2576" t="inlineStr">
@@ -25329,6 +25954,11 @@
           <t>TUNI047</t>
         </is>
       </c>
+      <c r="B2576" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2577">
       <c r="A2577" t="inlineStr">
@@ -25336,6 +25966,11 @@
           <t>TUNI048</t>
         </is>
       </c>
+      <c r="B2577" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2578">
       <c r="A2578" t="inlineStr">
@@ -25343,6 +25978,11 @@
           <t>TUNI053</t>
         </is>
       </c>
+      <c r="B2578" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2579">
       <c r="A2579" t="inlineStr">
@@ -25350,6 +25990,11 @@
           <t>TUNI054</t>
         </is>
       </c>
+      <c r="B2579" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2580">
       <c r="A2580" t="inlineStr">
@@ -25357,6 +26002,11 @@
           <t>TUNI055</t>
         </is>
       </c>
+      <c r="B2580" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2581">
       <c r="A2581" t="inlineStr">
@@ -25364,6 +26014,11 @@
           <t>TUNI056</t>
         </is>
       </c>
+      <c r="B2581" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2582">
       <c r="A2582" t="inlineStr">
@@ -25371,6 +26026,11 @@
           <t>TUNI059</t>
         </is>
       </c>
+      <c r="B2582" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2583">
       <c r="A2583" t="inlineStr">
@@ -25378,6 +26038,11 @@
           <t>TUNI060</t>
         </is>
       </c>
+      <c r="B2583" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2584">
       <c r="A2584" t="inlineStr">
@@ -25385,6 +26050,11 @@
           <t>TUNI062</t>
         </is>
       </c>
+      <c r="B2584" t="inlineStr">
+        <is>
+          <t>scaricato</t>
+        </is>
+      </c>
     </row>
     <row r="2585">
       <c r="A2585" t="inlineStr">
@@ -25425,6 +26095,11 @@
       <c r="A2590" t="inlineStr">
         <is>
           <t>ULHD001</t>
+        </is>
+      </c>
+      <c r="B2590" t="inlineStr">
+        <is>
+          <t>scaricato</t>
         </is>
       </c>
     </row>

</xml_diff>